<commit_message>
Keep only the latest 1.1.3 evaluation and simplify current reports
</commit_message>
<xml_diff>
--- a/docs/evaluation-mobile-v4-regression/Lifehub-Plus-V4-Regression.xlsx
+++ b/docs/evaluation-mobile-v4-regression/Lifehub-Plus-V4-Regression.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="回归结果" sheetId="1" r:id="R7cac80ee613d463e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中文120" sheetId="2" r:id="R35bbc9ac7c8b4354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English120" sheetId="3" r:id="Rfdb87567142b4625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="失败明细" sheetId="4" r:id="R741d8d7cb8a24110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="回归结果" sheetId="1" r:id="R3fe1883d19154e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中文120" sheetId="2" r:id="R955eb33c9ebc4782"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English120" sheetId="3" r:id="R4a5773ecbf6d4bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="失败明细" sheetId="4" r:id="Ra2f7cd7e78954a50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -429,7 +429,7 @@
   <x:sheetData>
     <x:row r="1" ht="27" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>Lifehub Plus v4 修复后复测</x:v>
+        <x:v>Lifehub Plus 1.1.3 测试结果</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -707,184 +707,171 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>首测与修复后比较</x:v>
+        <x:v>模块全部字段</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>首测通过</x:v>
+        <x:v>中文通过</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>首测总数</x:v>
+        <x:v>中文总数</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>首测比例</x:v>
+        <x:v>中文比例</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>复测通过</x:v>
+        <x:v>英文通过</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>复测总数</x:v>
+        <x:v>英文总数</x:v>
       </x:c>
       <x:c r="G13" s="12" t="str">
-        <x:v>复测比例</x:v>
+        <x:v>英文比例</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>比例变化</x:v>
+        <x:v>合计比例</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
       <x:c r="A14" s="1" t="str">
-        <x:v>模块分类</x:v>
+        <x:v>memo</x:v>
       </x:c>
       <x:c r="B14" s="1" t="n">
-        <x:v>188</x:v>
+        <x:f>SUMIF('中文120'!B4:B123,A14,'中文120'!K4:K123)</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C14" s="1" t="n">
-        <x:v>240</x:v>
+        <x:f>COUNTIF('中文120'!B4:B123,A14)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
         <x:f>B14/C14</x:f>
-        <x:v>0.7833333333333333</x:v>
+        <x:v>0.9666666666666667</x:v>
       </x:c>
       <x:c r="E14" s="1" t="n">
-        <x:f>B5+E5</x:f>
-        <x:v>240</x:v>
+        <x:f>SUMIF('English120'!B4:B123,A14,'English120'!K4:K123)</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F14" s="1" t="n">
-        <x:f>C5+F5</x:f>
-        <x:v>240</x:v>
+        <x:f>COUNTIF('English120'!B4:B123,A14)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G14" s="10" t="n">
         <x:f>E14/F14</x:f>
-        <x:v>1</x:v>
+        <x:v>0.9666666666666667</x:v>
       </x:c>
       <x:c r="H14" s="10" t="n">
-        <x:f>G14-D14</x:f>
-        <x:v>0.21666666666666667</x:v>
+        <x:f>(B14+E14)/(C14+F14)</x:f>
+        <x:v>0.9666666666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
       <x:c r="A15" s="1" t="str">
-        <x:v>必填字段</x:v>
+        <x:v>finance</x:v>
       </x:c>
       <x:c r="B15" s="1" t="n">
-        <x:v>398</x:v>
+        <x:f>SUMIF('中文120'!B4:B123,A15,'中文120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C15" s="1" t="n">
-        <x:v>432</x:v>
+        <x:f>COUNTIF('中文120'!B4:B123,A15)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
         <x:f>B15/C15</x:f>
-        <x:v>0.9212962962962963</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="1" t="n">
-        <x:f>B6+E6</x:f>
-        <x:v>432</x:v>
+        <x:f>SUMIF('English120'!B4:B123,A15,'English120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F15" s="1" t="n">
-        <x:f>C6+F6</x:f>
-        <x:v>432</x:v>
+        <x:f>COUNTIF('English120'!B4:B123,A15)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G15" s="10" t="n">
         <x:f>E15/F15</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H15" s="10" t="n">
-        <x:f>G15-D15</x:f>
-        <x:v>0.07870370370370372</x:v>
+        <x:f>(B15+E15)/(C15+F15)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
       <x:c r="A16" s="1" t="str">
-        <x:v>全部指定字段</x:v>
+        <x:v>schedule</x:v>
       </x:c>
       <x:c r="B16" s="1" t="n">
-        <x:v>153</x:v>
+        <x:f>SUMIF('中文120'!B4:B123,A16,'中文120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C16" s="1" t="n">
-        <x:v>240</x:v>
+        <x:f>COUNTIF('中文120'!B4:B123,A16)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
         <x:f>B16/C16</x:f>
-        <x:v>0.6375</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="1" t="n">
-        <x:f>B7+E7</x:f>
-        <x:v>238</x:v>
+        <x:f>SUMIF('English120'!B4:B123,A16,'English120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F16" s="1" t="n">
-        <x:f>C7+F7</x:f>
-        <x:v>240</x:v>
+        <x:f>COUNTIF('English120'!B4:B123,A16)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G16" s="10" t="n">
         <x:f>E16/F16</x:f>
-        <x:v>0.9916666666666667</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H16" s="10" t="n">
-        <x:f>G16-D16</x:f>
-        <x:v>0.35416666666666674</x:v>
+        <x:f>(B16+E16)/(C16+F16)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="27" customHeight="1">
       <x:c r="A17" s="1" t="str">
-        <x:v>支持请求草稿</x:v>
+        <x:v>health</x:v>
       </x:c>
       <x:c r="B17" s="1" t="n">
-        <x:v>123</x:v>
+        <x:f>SUMIF('中文120'!B4:B123,A17,'中文120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C17" s="1" t="n">
-        <x:v>180</x:v>
+        <x:f>COUNTIF('中文120'!B4:B123,A17)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
         <x:f>B17/C17</x:f>
-        <x:v>0.6833333333333333</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E17" s="1" t="n">
-        <x:f>B8+E8</x:f>
-        <x:v>178</x:v>
+        <x:f>SUMIF('English120'!B4:B123,A17,'English120'!K4:K123)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F17" s="1" t="n">
-        <x:f>C8+F8</x:f>
-        <x:v>180</x:v>
+        <x:f>COUNTIF('English120'!B4:B123,A17)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G17" s="10" t="n">
         <x:f>E17/F17</x:f>
-        <x:v>0.9888888888888889</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="10" t="n">
-        <x:f>G17-D17</x:f>
-        <x:v>0.3055555555555556</x:v>
+        <x:f>(B17+E17)/(C17+F17)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
-      <x:c r="A18" s="1" t="str">
-        <x:v>日期字段（含留空）</x:v>
-      </x:c>
-      <x:c r="B18" s="1" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="C18" s="1" t="n">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="D18" s="10" t="n">
-        <x:f>B18/C18</x:f>
-        <x:v>0.8888888888888888</x:v>
-      </x:c>
-      <x:c r="E18" s="1" t="n">
-        <x:f>B9+E9</x:f>
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="F18" s="1" t="n">
-        <x:f>C9+F9</x:f>
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="G18" s="10" t="n">
-        <x:f>E18/F18</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H18" s="10" t="n">
-        <x:f>G18-D18</x:f>
-        <x:v>0.11111111111111116</x:v>
-      </x:c>
+      <x:c r="A18" s="1"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1"/>
+      <x:c r="D18" s="1"/>
+      <x:c r="E18" s="1"/>
+      <x:c r="F18" s="1"/>
+      <x:c r="G18" s="1"/>
+      <x:c r="H18" s="1"/>
     </x:row>
     <x:row r="19" ht="27" customHeight="1">
       <x:c r="A19" s="1"/>
@@ -1002,7 +989,7 @@
     </x:row>
     <x:row r="28" ht="27" customHeight="1">
       <x:c r="A28" s="1" t="str">
-        <x:v>每条重新运行，单次尝试，不人工修正模型答案；原始首测数据与答案保持不变。</x:v>
+        <x:v>本表保留最新一次完整模型运行，每条单次尝试；原始输出和预期答案保持不变。</x:v>
       </x:c>
       <x:c r="B28" s="1"/>
       <x:c r="C28" s="1"/>
@@ -1113,7 +1100,7 @@
         <x:v>冻结版本</x:v>
       </x:c>
       <x:c r="B37" s="1" t="str">
-        <x:v>修复后的源文件 SHA-256 见协议；题目和原始首测保持不变</x:v>
+        <x:v>源文件 SHA-256 见协议；题目和当前原始输出保持不变</x:v>
       </x:c>
       <x:c r="C37" s="1"/>
       <x:c r="D37" s="1"/>
@@ -1127,7 +1114,7 @@
         <x:v>协议与哈希</x:v>
       </x:c>
       <x:c r="B38" s="1" t="str">
-        <x:v>原始首测：docs/evaluation-mobile-holdout-v4；本次：docs/evaluation-mobile-v4-regression</x:v>
+        <x:v>docs/evaluation-mobile-v4-regression/protocol.json 与 reproduction.json</x:v>
       </x:c>
       <x:c r="C38" s="1"/>
       <x:c r="D38" s="1"/>
@@ -9059,7 +9046,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f52022c5d34939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b01ce114a324730"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16938,7 +16925,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6ef49c0d834d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R587a51118bf14202"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17233,7 +17220,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720c571c165648f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0819c7c0d8f64d5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>